<commit_message>
niveles y balanceo inicial
</commit_message>
<xml_diff>
--- a/docs/Levels.xlsx
+++ b/docs/Levels.xlsx
@@ -79,6 +79,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -100,14 +101,21 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF6D"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -151,25 +159,41 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -181,6 +205,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF6D"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -295,201 +379,204 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.94"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="G2" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="5" t="n">
         <v>0.2</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="H3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="4" t="n">
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="5" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="H4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="I4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="J4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="B5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="H5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>4</v>
+      <c r="I5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="7" t="n">
         <v>2900</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="7" t="n">
         <v>3900</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="7" t="n">
         <v>4900</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="7" t="n">
         <v>5900</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="7" t="n">
         <v>6900</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="7" t="n">
         <v>8900</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="7" t="s">
         <v>14</v>
       </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>